<commit_message>
feat: improve and audit 2024 conversion quality
</commit_message>
<xml_diff>
--- a/data/2024/02-arad/9262-arad/budget_file.xlsx
+++ b/data/2024/02-arad/9262-arad/budget_file.xlsx
@@ -1685,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -1811,27 +1811,27 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Pagini asteptate</t>
+          <t>Linii anexe separate</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Pagini selectate</t>
+          <t>Celule numerice anexe separate</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Pagini procesate</t>
+          <t>Pagini asteptate</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1841,59 +1841,59 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>PDF complet</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>da</t>
-        </is>
+          <t>Pagini selectate</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Linii fara probleme</t>
+          <t>Pagini procesate</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>% curat</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>100</v>
+          <t>PDF complet</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Erori</t>
+          <t>Linii fara probleme</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Avertismente</t>
+          <t>% curat</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Informatii</t>
+          <t>Erori</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1903,53 +1903,49 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Schema publicare</t>
+          <t>Avertismente</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Bundle conversie</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>c5d84ebf152c5fe2d4e3d787</t>
-        </is>
+          <t>Informatii</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>SHA-256 sursa</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>9880703546e9dd3339932c6228ec8b67b4093184390ac6ea58b376cade181241</t>
-        </is>
+          <t>Schema publicare</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Format sursa</t>
+          <t>Bundle conversie</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>c5d84ebf152c5fe2d4e3d787</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>SHA-256 PDF sursa</t>
+          <t>SHA-256 sursa</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1961,10 +1957,34 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
+          <t>Format sursa</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>SHA-256 PDF sursa</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>9880703546e9dd3339932c6228ec8b67b4093184390ac6ea58b376cade181241</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
           <t>— Anexa (de la pagina 8)</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>local, pag. 8-10, 35 linii</t>
         </is>

</xml_diff>

<commit_message>
feat: improve and audit 2024 conversion quality (#20)
Co-authored-by: Dan Paraschiv <dan.paraschiv@gmail.com>
</commit_message>
<xml_diff>
--- a/data/2024/02-arad/9262-arad/budget_file.xlsx
+++ b/data/2024/02-arad/9262-arad/budget_file.xlsx
@@ -1685,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -1811,27 +1811,27 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Pagini asteptate</t>
+          <t>Linii anexe separate</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Pagini selectate</t>
+          <t>Celule numerice anexe separate</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Pagini procesate</t>
+          <t>Pagini asteptate</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1841,59 +1841,59 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>PDF complet</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>da</t>
-        </is>
+          <t>Pagini selectate</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Linii fara probleme</t>
+          <t>Pagini procesate</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>% curat</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>100</v>
+          <t>PDF complet</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Erori</t>
+          <t>Linii fara probleme</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Avertismente</t>
+          <t>% curat</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Informatii</t>
+          <t>Erori</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1903,53 +1903,49 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Schema publicare</t>
+          <t>Avertismente</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Bundle conversie</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>c5d84ebf152c5fe2d4e3d787</t>
-        </is>
+          <t>Informatii</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>SHA-256 sursa</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>9880703546e9dd3339932c6228ec8b67b4093184390ac6ea58b376cade181241</t>
-        </is>
+          <t>Schema publicare</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Format sursa</t>
+          <t>Bundle conversie</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>c5d84ebf152c5fe2d4e3d787</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>SHA-256 PDF sursa</t>
+          <t>SHA-256 sursa</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1961,10 +1957,34 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
+          <t>Format sursa</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>SHA-256 PDF sursa</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>9880703546e9dd3339932c6228ec8b67b4093184390ac6ea58b376cade181241</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
           <t>— Anexa (de la pagina 8)</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>local, pag. 8-10, 35 linii</t>
         </is>

</xml_diff>